<commit_message>
Release ATS OneBSS 0.9.25 with ticket ingest API
</commit_message>
<xml_diff>
--- a/Giao phiếu.xlsx
+++ b/Giao phiếu.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5FC4B15-1664-7846-B5BA-652050910A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C98996-55A3-0B44-963F-2F5A69CF7465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quy tắc giao phiếu" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="98">
   <si>
     <t>Nhóm 1</t>
   </si>
@@ -313,6 +326,9 @@
   </si>
   <si>
     <t>KTR-Đôi cáp quang</t>
+  </si>
+  <si>
+    <t>MyTV B2B</t>
   </si>
 </sst>
 </file>
@@ -780,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X66"/>
+  <dimension ref="A1:X67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="9" customWidth="1"/>
@@ -2401,16 +2417,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" s="11">
-        <v>25</v>
-      </c>
-      <c r="E40" s="13"/>
-      <c r="F40" s="10"/>
+        <v>17</v>
+      </c>
+      <c r="E40" s="12"/>
+      <c r="F40" s="11"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -2422,34 +2438,32 @@
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
-      <c r="R40" s="1"/>
-      <c r="S40" s="1"/>
-      <c r="T40" s="1"/>
-      <c r="U40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="V40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="W40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="X40" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="R40" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="S40" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="T40" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="U40" s="1"/>
+      <c r="V40" s="1"/>
+      <c r="W40" s="1"/>
+      <c r="X40" s="1"/>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A41" s="10">
         <v>39</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D41" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E41" s="13"/>
       <c r="F41" s="10"/>
@@ -2466,77 +2480,71 @@
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
-      <c r="T41" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="U41" s="1"/>
-      <c r="V41" s="1"/>
-      <c r="W41" s="1"/>
-      <c r="X41" s="1"/>
-    </row>
-    <row r="42" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T41" s="1"/>
+      <c r="U41" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="V41" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="W41" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="X41" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42" s="10">
         <v>40</v>
       </c>
-      <c r="B42" s="10" t="s">
-        <v>76</v>
+      <c r="B42" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="D42" s="11">
-        <v>17</v>
-      </c>
-      <c r="E42" s="12" t="s">
-        <v>47</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="E42" s="13"/>
       <c r="F42" s="10"/>
-      <c r="G42" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
-      <c r="L42" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="L42" s="1"/>
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
       <c r="O42" s="1"/>
-      <c r="P42" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q42" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="R42" s="10"/>
-      <c r="S42" s="10"/>
-      <c r="T42" s="10"/>
-      <c r="U42" s="10"/>
-      <c r="V42" s="10"/>
-      <c r="W42" s="10"/>
-      <c r="X42" s="10"/>
-    </row>
-    <row r="43" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P42" s="1"/>
+      <c r="Q42" s="1"/>
+      <c r="R42" s="1"/>
+      <c r="S42" s="1"/>
+      <c r="T42" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U42" s="1"/>
+      <c r="V42" s="1"/>
+      <c r="W42" s="1"/>
+      <c r="X42" s="1"/>
+    </row>
+    <row r="43" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10">
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C43" s="10" t="s">
-        <v>51</v>
+      <c r="C43" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D43" s="11">
-        <v>27</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="1" t="s">
@@ -2570,21 +2578,21 @@
       <c r="W43" s="10"/>
       <c r="X43" s="10"/>
     </row>
-    <row r="44" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="10">
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>46</v>
+        <v>76</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="D44" s="11">
-        <v>17</v>
-      </c>
-      <c r="E44" s="12" t="s">
-        <v>47</v>
+        <v>27</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F44" s="10"/>
       <c r="G44" s="1" t="s">
@@ -2618,21 +2626,21 @@
       <c r="W44" s="10"/>
       <c r="X44" s="10"/>
     </row>
-    <row r="45" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10">
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="C45" s="10" t="s">
-        <v>51</v>
+      <c r="C45" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D45" s="11">
-        <v>27</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F45" s="10"/>
       <c r="G45" s="1" t="s">
@@ -2666,21 +2674,21 @@
       <c r="W45" s="10"/>
       <c r="X45" s="10"/>
     </row>
-    <row r="46" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10">
         <v>44</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>49</v>
+        <v>77</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="D46" s="11">
-        <v>17</v>
-      </c>
-      <c r="E46" s="12" t="s">
-        <v>47</v>
+        <v>27</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F46" s="10"/>
       <c r="G46" s="1" t="s">
@@ -2714,7 +2722,7 @@
       <c r="W46" s="10"/>
       <c r="X46" s="10"/>
     </row>
-    <row r="47" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10">
         <v>45</v>
       </c>
@@ -2722,13 +2730,13 @@
         <v>78</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D47" s="11">
-        <v>27</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="1" t="s">
@@ -2762,21 +2770,21 @@
       <c r="W47" s="10"/>
       <c r="X47" s="10"/>
     </row>
-    <row r="48" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10">
         <v>46</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D48" s="11">
-        <v>17</v>
-      </c>
-      <c r="E48" s="12" t="s">
-        <v>47</v>
+        <v>27</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F48" s="10"/>
       <c r="G48" s="1" t="s">
@@ -2810,7 +2818,7 @@
       <c r="W48" s="10"/>
       <c r="X48" s="10"/>
     </row>
-    <row r="49" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10">
         <v>47</v>
       </c>
@@ -2818,13 +2826,13 @@
         <v>79</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D49" s="11">
-        <v>27</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F49" s="10"/>
       <c r="G49" s="1" t="s">
@@ -2858,21 +2866,21 @@
       <c r="W49" s="10"/>
       <c r="X49" s="10"/>
     </row>
-    <row r="50" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10">
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D50" s="11">
-        <v>17</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>47</v>
+        <v>27</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F50" s="10"/>
       <c r="G50" s="1" t="s">
@@ -2906,7 +2914,7 @@
       <c r="W50" s="10"/>
       <c r="X50" s="10"/>
     </row>
-    <row r="51" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10">
         <v>49</v>
       </c>
@@ -2914,13 +2922,13 @@
         <v>80</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D51" s="11">
-        <v>27</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F51" s="10"/>
       <c r="G51" s="1" t="s">
@@ -2954,43 +2962,45 @@
       <c r="W51" s="10"/>
       <c r="X51" s="10"/>
     </row>
-    <row r="52" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="10">
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C52" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D52" s="10">
-        <v>42</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>65</v>
+        <v>80</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D52" s="11">
+        <v>27</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="10"/>
-      <c r="J52" s="10"/>
-      <c r="K52" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L52" s="1"/>
-      <c r="M52" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N52" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="O52" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="P52" s="1"/>
+      <c r="G52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
+      <c r="L52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+      <c r="P52" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="Q52" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R52" s="10"/>
       <c r="S52" s="10"/>
@@ -3005,7 +3015,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C53" s="10" t="s">
         <v>64</v>
@@ -3051,7 +3061,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C54" s="10" t="s">
         <v>64</v>
@@ -3092,34 +3102,44 @@
       <c r="W54" s="10"/>
       <c r="X54" s="10"/>
     </row>
-    <row r="55" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10">
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="D55" s="10"/>
+        <v>64</v>
+      </c>
+      <c r="D55" s="10">
+        <v>42</v>
+      </c>
       <c r="E55" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="F55" s="10"/>
       <c r="G55" s="10"/>
       <c r="H55" s="10"/>
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
-      <c r="K55" s="10"/>
-      <c r="L55" s="10"/>
-      <c r="M55" s="10"/>
-      <c r="N55" s="10"/>
-      <c r="O55" s="10"/>
-      <c r="P55" s="10"/>
-      <c r="Q55" s="10"/>
+      <c r="K55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P55" s="1"/>
+      <c r="Q55" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="R55" s="10"/>
       <c r="S55" s="10"/>
       <c r="T55" s="10"/>
@@ -3128,46 +3148,34 @@
       <c r="W55" s="10"/>
       <c r="X55" s="10"/>
     </row>
-    <row r="56" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="10">
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D56" s="11">
-        <v>17</v>
-      </c>
-      <c r="E56" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F56" s="10"/>
-      <c r="G56" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J56" s="1"/>
-      <c r="K56" s="1"/>
-      <c r="L56" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M56" s="1"/>
-      <c r="N56" s="1"/>
-      <c r="O56" s="1"/>
-      <c r="P56" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q56" s="1" t="s">
-        <v>28</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D56" s="10"/>
+      <c r="E56" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10"/>
+      <c r="J56" s="10"/>
+      <c r="K56" s="10"/>
+      <c r="L56" s="10"/>
+      <c r="M56" s="10"/>
+      <c r="N56" s="10"/>
+      <c r="O56" s="10"/>
+      <c r="P56" s="10"/>
+      <c r="Q56" s="10"/>
       <c r="R56" s="10"/>
       <c r="S56" s="10"/>
       <c r="T56" s="10"/>
@@ -3176,21 +3184,21 @@
       <c r="W56" s="10"/>
       <c r="X56" s="10"/>
     </row>
-    <row r="57" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="10">
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C57" s="10" t="s">
-        <v>51</v>
+      <c r="C57" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D57" s="11">
-        <v>27</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F57" s="10"/>
       <c r="G57" s="1" t="s">
@@ -3224,21 +3232,21 @@
       <c r="W57" s="10"/>
       <c r="X57" s="10"/>
     </row>
-    <row r="58" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="10">
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>46</v>
+        <v>86</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="D58" s="11">
-        <v>17</v>
-      </c>
-      <c r="E58" s="12" t="s">
-        <v>47</v>
+        <v>27</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F58" s="10"/>
       <c r="G58" s="1" t="s">
@@ -3272,21 +3280,21 @@
       <c r="W58" s="10"/>
       <c r="X58" s="10"/>
     </row>
-    <row r="59" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="10">
         <v>57</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="C59" s="10" t="s">
-        <v>51</v>
+      <c r="C59" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D59" s="11">
-        <v>27</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E59" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F59" s="10"/>
       <c r="G59" s="1" t="s">
@@ -3320,43 +3328,45 @@
       <c r="W59" s="10"/>
       <c r="X59" s="10"/>
     </row>
-    <row r="60" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="10">
         <v>58</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D60" s="10">
-        <v>42</v>
-      </c>
-      <c r="E60" s="13" t="s">
-        <v>65</v>
+        <v>51</v>
+      </c>
+      <c r="D60" s="11">
+        <v>27</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
-      <c r="K60" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L60" s="1"/>
-      <c r="M60" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N60" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="O60" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="P60" s="1"/>
+      <c r="G60" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1"/>
+      <c r="O60" s="1"/>
+      <c r="P60" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="Q60" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R60" s="10"/>
       <c r="S60" s="10"/>
@@ -3366,45 +3376,43 @@
       <c r="W60" s="10"/>
       <c r="X60" s="10"/>
     </row>
-    <row r="61" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="10">
         <v>59</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D61" s="11">
-        <v>17</v>
-      </c>
-      <c r="E61" s="12" t="s">
-        <v>47</v>
+        <v>88</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D61" s="10">
+        <v>42</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>65</v>
       </c>
       <c r="F61" s="10"/>
-      <c r="G61" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I61" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J61" s="1"/>
-      <c r="K61" s="1"/>
-      <c r="L61" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M61" s="1"/>
-      <c r="N61" s="1"/>
-      <c r="O61" s="1"/>
-      <c r="P61" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
+      <c r="I61" s="10"/>
+      <c r="J61" s="10"/>
+      <c r="K61" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L61" s="1"/>
+      <c r="M61" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N61" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O61" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P61" s="1"/>
       <c r="Q61" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R61" s="10"/>
       <c r="S61" s="10"/>
@@ -3414,21 +3422,21 @@
       <c r="W61" s="10"/>
       <c r="X61" s="10"/>
     </row>
-    <row r="62" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="10">
         <v>60</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C62" s="10" t="s">
-        <v>51</v>
+      <c r="C62" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="D62" s="11">
-        <v>27</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E62" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F62" s="10"/>
       <c r="G62" s="1" t="s">
@@ -3462,34 +3470,46 @@
       <c r="W62" s="10"/>
       <c r="X62" s="10"/>
     </row>
-    <row r="63" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="10">
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D63" s="10"/>
-      <c r="E63" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
-      <c r="M63" s="10"/>
-      <c r="N63" s="10"/>
-      <c r="O63" s="10"/>
-      <c r="P63" s="10"/>
-      <c r="Q63" s="10"/>
+        <v>51</v>
+      </c>
+      <c r="D63" s="11">
+        <v>27</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F63" s="10"/>
+      <c r="G63" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="L63" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M63" s="1"/>
+      <c r="N63" s="1"/>
+      <c r="O63" s="1"/>
+      <c r="P63" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q63" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="R63" s="10"/>
       <c r="S63" s="10"/>
       <c r="T63" s="10"/>
@@ -3498,75 +3518,65 @@
       <c r="W63" s="10"/>
       <c r="X63" s="10"/>
     </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="10">
         <v>62</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="D64" s="11">
-        <v>17</v>
-      </c>
-      <c r="E64" s="12"/>
-      <c r="F64" s="11"/>
-      <c r="G64" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I64" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J64" s="1"/>
-      <c r="K64" s="1"/>
-      <c r="L64" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M64" s="1"/>
-      <c r="N64" s="1"/>
-      <c r="O64" s="1"/>
-      <c r="P64" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q64" s="1"/>
-      <c r="R64" s="1"/>
-      <c r="S64" s="1"/>
-      <c r="T64" s="1"/>
-      <c r="U64" s="1"/>
-      <c r="V64" s="1"/>
-      <c r="W64" s="1"/>
-      <c r="X64" s="1"/>
-    </row>
-    <row r="65" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+      <c r="D64" s="10"/>
+      <c r="E64" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G64" s="10"/>
+      <c r="H64" s="10"/>
+      <c r="I64" s="10"/>
+      <c r="J64" s="10"/>
+      <c r="K64" s="10"/>
+      <c r="L64" s="10"/>
+      <c r="M64" s="10"/>
+      <c r="N64" s="10"/>
+      <c r="O64" s="10"/>
+      <c r="P64" s="10"/>
+      <c r="Q64" s="10"/>
+      <c r="R64" s="10"/>
+      <c r="S64" s="10"/>
+      <c r="T64" s="10"/>
+      <c r="U64" s="10"/>
+      <c r="V64" s="10"/>
+      <c r="W64" s="10"/>
+      <c r="X64" s="10"/>
+    </row>
+    <row r="65" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A65" s="10">
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="D65" s="11">
         <v>17</v>
       </c>
-      <c r="E65" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F65" s="10"/>
+      <c r="E65" s="12"/>
+      <c r="F65" s="11"/>
       <c r="G65" s="1" t="s">
         <v>27</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
@@ -3579,18 +3589,16 @@
       <c r="P65" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q65" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="R65" s="10"/>
-      <c r="S65" s="10"/>
-      <c r="T65" s="10"/>
-      <c r="U65" s="10"/>
-      <c r="V65" s="10"/>
-      <c r="W65" s="10"/>
-      <c r="X65" s="10"/>
-    </row>
-    <row r="66" spans="1:24" ht="54" x14ac:dyDescent="0.2">
+      <c r="Q65" s="1"/>
+      <c r="R65" s="1"/>
+      <c r="S65" s="1"/>
+      <c r="T65" s="1"/>
+      <c r="U65" s="1"/>
+      <c r="V65" s="1"/>
+      <c r="W65" s="1"/>
+      <c r="X65" s="1"/>
+    </row>
+    <row r="66" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A66" s="10">
         <v>64</v>
       </c>
@@ -3598,13 +3606,13 @@
         <v>96</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D66" s="11">
-        <v>27</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>52</v>
+        <v>17</v>
+      </c>
+      <c r="E66" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="F66" s="10"/>
       <c r="G66" s="1" t="s">
@@ -3637,6 +3645,54 @@
       <c r="V66" s="10"/>
       <c r="W66" s="10"/>
       <c r="X66" s="10"/>
+    </row>
+    <row r="67" spans="1:24" ht="54" x14ac:dyDescent="0.2">
+      <c r="A67" s="10">
+        <v>65</v>
+      </c>
+      <c r="B67" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C67" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D67" s="11">
+        <v>27</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F67" s="10"/>
+      <c r="G67" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J67" s="1"/>
+      <c r="K67" s="1"/>
+      <c r="L67" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M67" s="1"/>
+      <c r="N67" s="1"/>
+      <c r="O67" s="1"/>
+      <c r="P67" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q67" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="R67" s="10"/>
+      <c r="S67" s="10"/>
+      <c r="T67" s="10"/>
+      <c r="U67" s="10"/>
+      <c r="V67" s="10"/>
+      <c r="W67" s="10"/>
+      <c r="X67" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add per-service API opt-in from workbook
</commit_message>
<xml_diff>
--- a/Giao phiếu.xlsx
+++ b/Giao phiếu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C98996-55A3-0B44-963F-2F5A69CF7465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1D8A89-4A1E-E64D-AD8D-543FF9690CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="100">
   <si>
     <t>Nhóm 1</t>
   </si>
@@ -329,6 +329,12 @@
   </si>
   <si>
     <t>MyTV B2B</t>
+  </si>
+  <si>
+    <t>Gửi API</t>
+  </si>
+  <si>
+    <t>Có</t>
   </si>
 </sst>
 </file>
@@ -796,7 +802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X67"/>
+  <dimension ref="A1:Y67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="9" customWidth="1"/>
@@ -827,7 +833,7 @@
     <col min="26" max="16384" width="10.83203125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="F1" s="15" t="s">
         <v>0</v>
       </c>
@@ -852,7 +858,7 @@
       <c r="W1" s="16"/>
       <c r="X1" s="17"/>
     </row>
-    <row r="2" spans="1:24" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:25" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -925,8 +931,11 @@
       <c r="X2" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y2" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="10">
         <v>1</v>
       </c>
@@ -965,8 +974,9 @@
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y3" s="10"/>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" s="10">
         <v>2</v>
       </c>
@@ -1003,8 +1013,9 @@
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y4" s="10"/>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" s="10">
         <v>3</v>
       </c>
@@ -1041,8 +1052,9 @@
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y5" s="10"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6" s="10">
         <v>4</v>
       </c>
@@ -1077,8 +1089,9 @@
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y6" s="10"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="10">
         <v>5</v>
       </c>
@@ -1113,8 +1126,9 @@
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y7" s="10"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" s="10">
         <v>6</v>
       </c>
@@ -1151,8 +1165,9 @@
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y8" s="10"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="10">
         <v>7</v>
       </c>
@@ -1195,8 +1210,11 @@
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
       <c r="X9" s="1"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y9" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" s="10">
         <v>8</v>
       </c>
@@ -1235,8 +1253,9 @@
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
       <c r="X10" s="1"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y10" s="10"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="10">
         <v>9</v>
       </c>
@@ -1275,8 +1294,9 @@
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y11" s="10"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12" s="10">
         <v>10</v>
       </c>
@@ -1315,8 +1335,9 @@
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y12" s="10"/>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
         <v>11</v>
       </c>
@@ -1355,8 +1376,9 @@
       <c r="V13" s="1"/>
       <c r="W13" s="1"/>
       <c r="X13" s="1"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y13" s="10"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
         <v>12</v>
       </c>
@@ -1395,8 +1417,9 @@
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
       <c r="X14" s="1"/>
-    </row>
-    <row r="15" spans="1:24" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y14" s="10"/>
+    </row>
+    <row r="15" spans="1:25" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>13</v>
       </c>
@@ -1439,8 +1462,9 @@
       <c r="X15" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y15" s="10"/>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
         <v>14</v>
       </c>
@@ -1477,8 +1501,9 @@
       <c r="V16" s="1"/>
       <c r="W16" s="1"/>
       <c r="X16" s="1"/>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y16" s="10"/>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
         <v>15</v>
       </c>
@@ -1515,8 +1540,9 @@
       <c r="V17" s="1"/>
       <c r="W17" s="1"/>
       <c r="X17" s="1"/>
-    </row>
-    <row r="18" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y17" s="10"/>
+    </row>
+    <row r="18" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
         <v>16</v>
       </c>
@@ -1563,8 +1589,11 @@
       <c r="V18" s="1"/>
       <c r="W18" s="1"/>
       <c r="X18" s="1"/>
-    </row>
-    <row r="19" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y18" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
         <v>17</v>
       </c>
@@ -1611,8 +1640,11 @@
       <c r="V19" s="1"/>
       <c r="W19" s="1"/>
       <c r="X19" s="1"/>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y19" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
         <v>18</v>
       </c>
@@ -1655,8 +1687,11 @@
       <c r="V20" s="1"/>
       <c r="W20" s="1"/>
       <c r="X20" s="1"/>
-    </row>
-    <row r="21" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y20" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>19</v>
       </c>
@@ -1703,8 +1738,11 @@
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
       <c r="X21" s="1"/>
-    </row>
-    <row r="22" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y21" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
         <v>20</v>
       </c>
@@ -1751,8 +1789,11 @@
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y22" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
         <v>21</v>
       </c>
@@ -1787,8 +1828,9 @@
       <c r="V23" s="1"/>
       <c r="W23" s="1"/>
       <c r="X23" s="1"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y23" s="10"/>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
         <v>22</v>
       </c>
@@ -1825,8 +1867,9 @@
       <c r="V24" s="1"/>
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y24" s="10"/>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
         <v>23</v>
       </c>
@@ -1863,8 +1906,9 @@
       <c r="V25" s="1"/>
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y25" s="10"/>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
         <v>24</v>
       </c>
@@ -1901,8 +1945,9 @@
       <c r="V26" s="1"/>
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y26" s="10"/>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A27" s="10">
         <v>25</v>
       </c>
@@ -1939,8 +1984,9 @@
       <c r="V27" s="1"/>
       <c r="W27" s="1"/>
       <c r="X27" s="1"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y27" s="10"/>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A28" s="10">
         <v>26</v>
       </c>
@@ -1975,8 +2021,9 @@
       <c r="V28" s="1"/>
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y28" s="10"/>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
         <v>27</v>
       </c>
@@ -2013,8 +2060,9 @@
       <c r="V29" s="1"/>
       <c r="W29" s="1"/>
       <c r="X29" s="1"/>
-    </row>
-    <row r="30" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y29" s="10"/>
+    </row>
+    <row r="30" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
         <v>28</v>
       </c>
@@ -2059,8 +2107,11 @@
       <c r="V30" s="1"/>
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
-    </row>
-    <row r="31" spans="1:24" ht="90" x14ac:dyDescent="0.2">
+      <c r="Y30" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" ht="90" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
         <v>29</v>
       </c>
@@ -2099,8 +2150,9 @@
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
-    </row>
-    <row r="32" spans="1:24" ht="90" x14ac:dyDescent="0.2">
+      <c r="Y31" s="10"/>
+    </row>
+    <row r="32" spans="1:25" ht="90" x14ac:dyDescent="0.2">
       <c r="A32" s="10">
         <v>30</v>
       </c>
@@ -2139,8 +2191,9 @@
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>
-    </row>
-    <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y32" s="10"/>
+    </row>
+    <row r="33" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="10">
         <v>31</v>
       </c>
@@ -2179,8 +2232,9 @@
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
       <c r="X33" s="1"/>
-    </row>
-    <row r="34" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y33" s="10"/>
+    </row>
+    <row r="34" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="10">
         <v>32</v>
       </c>
@@ -2219,8 +2273,9 @@
       <c r="V34" s="1"/>
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
-    </row>
-    <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y34" s="10"/>
+    </row>
+    <row r="35" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="10">
         <v>33</v>
       </c>
@@ -2257,8 +2312,9 @@
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
       <c r="X35" s="1"/>
-    </row>
-    <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y35" s="10"/>
+    </row>
+    <row r="36" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="10">
         <v>34</v>
       </c>
@@ -2295,8 +2351,9 @@
       <c r="V36" s="1"/>
       <c r="W36" s="1"/>
       <c r="X36" s="1"/>
-    </row>
-    <row r="37" spans="1:24" ht="36" x14ac:dyDescent="0.2">
+      <c r="Y36" s="10"/>
+    </row>
+    <row r="37" spans="1:25" ht="36" x14ac:dyDescent="0.2">
       <c r="A37" s="10">
         <v>35</v>
       </c>
@@ -2333,8 +2390,9 @@
       <c r="V37" s="1"/>
       <c r="W37" s="1"/>
       <c r="X37" s="1"/>
-    </row>
-    <row r="38" spans="1:24" ht="36" x14ac:dyDescent="0.2">
+      <c r="Y37" s="10"/>
+    </row>
+    <row r="38" spans="1:25" ht="36" x14ac:dyDescent="0.2">
       <c r="A38" s="10">
         <v>36</v>
       </c>
@@ -2371,8 +2429,9 @@
       <c r="V38" s="1"/>
       <c r="W38" s="1"/>
       <c r="X38" s="1"/>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y38" s="10"/>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A39" s="10">
         <v>37</v>
       </c>
@@ -2411,8 +2470,9 @@
       <c r="V39" s="1"/>
       <c r="W39" s="1"/>
       <c r="X39" s="1"/>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y39" s="10"/>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A40" s="10">
         <v>38</v>
       </c>
@@ -2451,8 +2511,9 @@
       <c r="V40" s="1"/>
       <c r="W40" s="1"/>
       <c r="X40" s="1"/>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y40" s="10"/>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A41" s="10">
         <v>39</v>
       </c>
@@ -2493,8 +2554,9 @@
       <c r="X41" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y41" s="10"/>
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A42" s="10">
         <v>40</v>
       </c>
@@ -2529,8 +2591,9 @@
       <c r="V42" s="1"/>
       <c r="W42" s="1"/>
       <c r="X42" s="1"/>
-    </row>
-    <row r="43" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y42" s="10"/>
+    </row>
+    <row r="43" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10">
         <v>41</v>
       </c>
@@ -2577,8 +2640,11 @@
       <c r="V43" s="10"/>
       <c r="W43" s="10"/>
       <c r="X43" s="10"/>
-    </row>
-    <row r="44" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y43" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="10">
         <v>42</v>
       </c>
@@ -2625,8 +2691,11 @@
       <c r="V44" s="10"/>
       <c r="W44" s="10"/>
       <c r="X44" s="10"/>
-    </row>
-    <row r="45" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y44" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10">
         <v>43</v>
       </c>
@@ -2673,8 +2742,11 @@
       <c r="V45" s="10"/>
       <c r="W45" s="10"/>
       <c r="X45" s="10"/>
-    </row>
-    <row r="46" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y45" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10">
         <v>44</v>
       </c>
@@ -2721,8 +2793,11 @@
       <c r="V46" s="10"/>
       <c r="W46" s="10"/>
       <c r="X46" s="10"/>
-    </row>
-    <row r="47" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y46" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10">
         <v>45</v>
       </c>
@@ -2769,8 +2844,11 @@
       <c r="V47" s="10"/>
       <c r="W47" s="10"/>
       <c r="X47" s="10"/>
-    </row>
-    <row r="48" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y47" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10">
         <v>46</v>
       </c>
@@ -2817,8 +2895,11 @@
       <c r="V48" s="10"/>
       <c r="W48" s="10"/>
       <c r="X48" s="10"/>
-    </row>
-    <row r="49" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y48" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10">
         <v>47</v>
       </c>
@@ -2865,8 +2946,11 @@
       <c r="V49" s="10"/>
       <c r="W49" s="10"/>
       <c r="X49" s="10"/>
-    </row>
-    <row r="50" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y49" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10">
         <v>48</v>
       </c>
@@ -2913,8 +2997,11 @@
       <c r="V50" s="10"/>
       <c r="W50" s="10"/>
       <c r="X50" s="10"/>
-    </row>
-    <row r="51" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y50" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10">
         <v>49</v>
       </c>
@@ -2961,8 +3048,11 @@
       <c r="V51" s="10"/>
       <c r="W51" s="10"/>
       <c r="X51" s="10"/>
-    </row>
-    <row r="52" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y51" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="10">
         <v>50</v>
       </c>
@@ -3009,8 +3099,11 @@
       <c r="V52" s="10"/>
       <c r="W52" s="10"/>
       <c r="X52" s="10"/>
-    </row>
-    <row r="53" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y52" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10">
         <v>51</v>
       </c>
@@ -3055,8 +3148,11 @@
       <c r="V53" s="10"/>
       <c r="W53" s="10"/>
       <c r="X53" s="10"/>
-    </row>
-    <row r="54" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y53" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="54" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="10">
         <v>52</v>
       </c>
@@ -3101,8 +3197,11 @@
       <c r="V54" s="10"/>
       <c r="W54" s="10"/>
       <c r="X54" s="10"/>
-    </row>
-    <row r="55" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y54" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="55" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10">
         <v>53</v>
       </c>
@@ -3147,8 +3246,11 @@
       <c r="V55" s="10"/>
       <c r="W55" s="10"/>
       <c r="X55" s="10"/>
-    </row>
-    <row r="56" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y55" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="56" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="10">
         <v>54</v>
       </c>
@@ -3183,8 +3285,9 @@
       <c r="V56" s="10"/>
       <c r="W56" s="10"/>
       <c r="X56" s="10"/>
-    </row>
-    <row r="57" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y56" s="10"/>
+    </row>
+    <row r="57" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="10">
         <v>55</v>
       </c>
@@ -3231,8 +3334,11 @@
       <c r="V57" s="10"/>
       <c r="W57" s="10"/>
       <c r="X57" s="10"/>
-    </row>
-    <row r="58" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y57" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="58" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="10">
         <v>56</v>
       </c>
@@ -3279,8 +3385,11 @@
       <c r="V58" s="10"/>
       <c r="W58" s="10"/>
       <c r="X58" s="10"/>
-    </row>
-    <row r="59" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y58" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="59" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="10">
         <v>57</v>
       </c>
@@ -3327,8 +3436,11 @@
       <c r="V59" s="10"/>
       <c r="W59" s="10"/>
       <c r="X59" s="10"/>
-    </row>
-    <row r="60" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y59" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="60" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="10">
         <v>58</v>
       </c>
@@ -3375,8 +3487,11 @@
       <c r="V60" s="10"/>
       <c r="W60" s="10"/>
       <c r="X60" s="10"/>
-    </row>
-    <row r="61" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y60" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="61" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="10">
         <v>59</v>
       </c>
@@ -3421,8 +3536,11 @@
       <c r="V61" s="10"/>
       <c r="W61" s="10"/>
       <c r="X61" s="10"/>
-    </row>
-    <row r="62" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y61" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="62" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="10">
         <v>60</v>
       </c>
@@ -3469,8 +3587,11 @@
       <c r="V62" s="10"/>
       <c r="W62" s="10"/>
       <c r="X62" s="10"/>
-    </row>
-    <row r="63" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y62" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="63" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="10">
         <v>61</v>
       </c>
@@ -3517,8 +3638,11 @@
       <c r="V63" s="10"/>
       <c r="W63" s="10"/>
       <c r="X63" s="10"/>
-    </row>
-    <row r="64" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Y63" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="64" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="10">
         <v>62</v>
       </c>
@@ -3553,8 +3677,9 @@
       <c r="V64" s="10"/>
       <c r="W64" s="10"/>
       <c r="X64" s="10"/>
-    </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y64" s="10"/>
+    </row>
+    <row r="65" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A65" s="10">
         <v>63</v>
       </c>
@@ -3597,8 +3722,11 @@
       <c r="V65" s="1"/>
       <c r="W65" s="1"/>
       <c r="X65" s="1"/>
-    </row>
-    <row r="66" spans="1:24" ht="18" x14ac:dyDescent="0.2">
+      <c r="Y65" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="66" spans="1:25" ht="18" x14ac:dyDescent="0.2">
       <c r="A66" s="10">
         <v>64</v>
       </c>
@@ -3645,8 +3773,11 @@
       <c r="V66" s="10"/>
       <c r="W66" s="10"/>
       <c r="X66" s="10"/>
-    </row>
-    <row r="67" spans="1:24" ht="54" x14ac:dyDescent="0.2">
+      <c r="Y66" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="67" spans="1:25" ht="54" x14ac:dyDescent="0.2">
       <c r="A67" s="10">
         <v>65</v>
       </c>
@@ -3693,6 +3824,9 @@
       <c r="V67" s="10"/>
       <c r="W67" s="10"/>
       <c r="X67" s="10"/>
+      <c r="Y67" s="10" t="s">
+        <v>99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Release ATS OneBSS 0.9.30 with browser tab order update
</commit_message>
<xml_diff>
--- a/Giao phiếu.xlsx
+++ b/Giao phiếu.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1D8A89-4A1E-E64D-AD8D-543FF9690CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1039D6B4-37E7-1A40-9801-A7E45B844613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quy tắc giao phiếu" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="100">
   <si>
     <t>Nhóm 1</t>
   </si>
@@ -1202,7 +1202,9 @@
       <c r="P9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q9" s="1"/>
+      <c r="Q9" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
@@ -1580,7 +1582,7 @@
         <v>27</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -1631,7 +1633,7 @@
         <v>27</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -1677,9 +1679,7 @@
         <v>27</v>
       </c>
       <c r="P20" s="1"/>
-      <c r="Q20" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
@@ -1729,7 +1729,7 @@
         <v>27</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
@@ -1780,7 +1780,7 @@
         <v>27</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
@@ -2097,9 +2097,7 @@
         <v>27</v>
       </c>
       <c r="P30" s="1"/>
-      <c r="Q30" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
@@ -2631,7 +2629,7 @@
         <v>27</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R43" s="10"/>
       <c r="S43" s="10"/>
@@ -2682,7 +2680,7 @@
         <v>27</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R44" s="10"/>
       <c r="S44" s="10"/>
@@ -2733,7 +2731,7 @@
         <v>27</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R45" s="10"/>
       <c r="S45" s="10"/>
@@ -2784,7 +2782,7 @@
         <v>27</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R46" s="10"/>
       <c r="S46" s="10"/>
@@ -2835,7 +2833,7 @@
         <v>27</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R47" s="10"/>
       <c r="S47" s="10"/>
@@ -2886,7 +2884,7 @@
         <v>27</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R48" s="10"/>
       <c r="S48" s="10"/>
@@ -2937,7 +2935,7 @@
         <v>27</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R49" s="10"/>
       <c r="S49" s="10"/>
@@ -2988,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R50" s="10"/>
       <c r="S50" s="10"/>
@@ -3039,7 +3037,7 @@
         <v>27</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R51" s="10"/>
       <c r="S51" s="10"/>
@@ -3090,7 +3088,7 @@
         <v>27</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R52" s="10"/>
       <c r="S52" s="10"/>
@@ -3138,9 +3136,7 @@
         <v>27</v>
       </c>
       <c r="P53" s="1"/>
-      <c r="Q53" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q53" s="1"/>
       <c r="R53" s="10"/>
       <c r="S53" s="10"/>
       <c r="T53" s="10"/>
@@ -3187,9 +3183,7 @@
         <v>27</v>
       </c>
       <c r="P54" s="1"/>
-      <c r="Q54" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q54" s="1"/>
       <c r="R54" s="10"/>
       <c r="S54" s="10"/>
       <c r="T54" s="10"/>
@@ -3236,9 +3230,7 @@
         <v>27</v>
       </c>
       <c r="P55" s="1"/>
-      <c r="Q55" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q55" s="1"/>
       <c r="R55" s="10"/>
       <c r="S55" s="10"/>
       <c r="T55" s="10"/>
@@ -3325,7 +3317,7 @@
         <v>27</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R57" s="10"/>
       <c r="S57" s="10"/>
@@ -3376,7 +3368,7 @@
         <v>27</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R58" s="10"/>
       <c r="S58" s="10"/>
@@ -3427,7 +3419,7 @@
         <v>27</v>
       </c>
       <c r="Q59" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R59" s="10"/>
       <c r="S59" s="10"/>
@@ -3478,7 +3470,7 @@
         <v>27</v>
       </c>
       <c r="Q60" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R60" s="10"/>
       <c r="S60" s="10"/>
@@ -3526,9 +3518,7 @@
         <v>27</v>
       </c>
       <c r="P61" s="1"/>
-      <c r="Q61" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q61" s="1"/>
       <c r="R61" s="10"/>
       <c r="S61" s="10"/>
       <c r="T61" s="10"/>
@@ -3578,7 +3568,7 @@
         <v>27</v>
       </c>
       <c r="Q62" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R62" s="10"/>
       <c r="S62" s="10"/>
@@ -3629,7 +3619,7 @@
         <v>27</v>
       </c>
       <c r="Q63" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R63" s="10"/>
       <c r="S63" s="10"/>
@@ -3714,7 +3704,9 @@
       <c r="P65" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q65" s="1"/>
+      <c r="Q65" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="R65" s="1"/>
       <c r="S65" s="1"/>
       <c r="T65" s="1"/>
@@ -3764,7 +3756,7 @@
         <v>27</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R66" s="10"/>
       <c r="S66" s="10"/>
@@ -3815,7 +3807,7 @@
         <v>27</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R67" s="10"/>
       <c r="S67" s="10"/>

</xml_diff>

<commit_message>
Release ATS OneBSS 0.9.33 with weighted service rules
</commit_message>
<xml_diff>
--- a/Giao phiếu.xlsx
+++ b/Giao phiếu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1039D6B4-37E7-1A40-9801-A7E45B844613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{505F5632-7BB2-664B-964D-4EB8BA9F7EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quy tắc giao phiếu" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="99">
   <si>
     <t>Nhóm 1</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>Lê Đức Vinh</t>
-  </si>
-  <si>
-    <t>Ngọc Thành Kiên</t>
   </si>
   <si>
     <t>Nguyễn Hoàng Dương</t>
@@ -802,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y67"/>
+  <dimension ref="A1:X67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="9" customWidth="1"/>
@@ -822,18 +819,17 @@
     <col min="15" max="15" width="16" style="9" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="18" style="9" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11" style="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.1640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.83203125" style="9" customWidth="1"/>
-    <col min="26" max="16384" width="10.83203125" style="9"/>
+    <col min="18" max="18" width="18.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.1640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11" style="9" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.1640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.1640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.1640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.83203125" style="9" customWidth="1"/>
+    <col min="25" max="16384" width="10.83203125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="F1" s="15" t="s">
         <v>0</v>
       </c>
@@ -849,16 +845,15 @@
       <c r="P1" s="16"/>
       <c r="Q1" s="16"/>
       <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="17"/>
-      <c r="U1" s="15" t="s">
+      <c r="S1" s="17"/>
+      <c r="T1" s="15" t="s">
         <v>1</v>
       </c>
+      <c r="U1" s="16"/>
       <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="17"/>
-    </row>
-    <row r="2" spans="1:25" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W1" s="17"/>
+    </row>
+    <row r="2" spans="1:24" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -928,22 +923,19 @@
       <c r="W2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="X2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y2" s="10" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X2" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" s="10">
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D3" s="11">
         <v>10</v>
@@ -965,26 +957,25 @@
         <v>27</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
-      <c r="X3" s="1"/>
-      <c r="Y3" s="10"/>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X3" s="10"/>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="10">
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="11">
         <v>17</v>
@@ -1005,25 +996,24 @@
       <c r="R4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="S4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="T4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="10"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X4" s="10"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="10">
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D5" s="11">
         <v>17</v>
@@ -1044,25 +1034,24 @@
       <c r="R5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="S5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="T5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="10"/>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X5" s="10"/>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="10">
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>32</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>33</v>
       </c>
       <c r="D6" s="11">
         <v>10</v>
@@ -1070,7 +1059,7 @@
       <c r="E6" s="12"/>
       <c r="F6" s="11"/>
       <c r="G6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -1088,18 +1077,17 @@
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="10"/>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X6" s="10"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="10">
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7" s="11">
         <v>10</v>
@@ -1107,7 +1095,7 @@
       <c r="E7" s="12"/>
       <c r="F7" s="11"/>
       <c r="G7" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -1125,18 +1113,17 @@
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="10"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X7" s="10"/>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="10">
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D8" s="11">
         <v>17</v>
@@ -1157,25 +1144,24 @@
       <c r="R8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="S8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="T8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="10"/>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X8" s="10"/>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="10">
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D9" s="11">
         <v>17</v>
@@ -1183,27 +1169,27 @@
       <c r="E9" s="12"/>
       <c r="F9" s="11"/>
       <c r="G9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -1211,20 +1197,19 @@
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X9" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="10">
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10" s="11">
         <v>17</v>
@@ -1246,26 +1231,25 @@
         <v>27</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
-      <c r="X10" s="1"/>
-      <c r="Y10" s="10"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X10" s="10"/>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="10">
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" s="11">
         <v>17</v>
@@ -1287,26 +1271,25 @@
         <v>27</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
-      <c r="X11" s="1"/>
-      <c r="Y11" s="10"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X11" s="10"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="10">
         <v>10</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D12" s="11">
         <v>17</v>
@@ -1328,18 +1311,17 @@
         <v>27</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
-      <c r="X12" s="1"/>
-      <c r="Y12" s="10"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X12" s="10"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
         <v>11</v>
       </c>
@@ -1347,7 +1329,7 @@
         <v>1800</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D13" s="11">
         <v>17</v>
@@ -1369,18 +1351,17 @@
         <v>27</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="1"/>
-      <c r="Y13" s="10"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X13" s="10"/>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
         <v>12</v>
       </c>
@@ -1388,7 +1369,7 @@
         <v>1900</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D14" s="11">
         <v>17</v>
@@ -1410,32 +1391,31 @@
         <v>27</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
-      <c r="X14" s="1"/>
-      <c r="Y14" s="10"/>
-    </row>
-    <row r="15" spans="1:25" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X14" s="10"/>
+    </row>
+    <row r="15" spans="1:24" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>13</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D15" s="11">
         <v>20</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="1"/>
@@ -1451,30 +1431,29 @@
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
-      <c r="T15" s="1"/>
+      <c r="T15" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="U15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="X15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y15" s="10"/>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+      <c r="X15" s="10"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
         <v>14</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D16" s="11">
         <v>17</v>
@@ -1482,11 +1461,11 @@
       <c r="E16" s="12"/>
       <c r="F16" s="11"/>
       <c r="G16" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1502,18 +1481,17 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="W16" s="1"/>
-      <c r="X16" s="1"/>
-      <c r="Y16" s="10"/>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X16" s="10"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
         <v>15</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17" s="11">
         <v>17</v>
@@ -1521,12 +1499,12 @@
       <c r="E17" s="12"/>
       <c r="F17" s="11"/>
       <c r="G17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
@@ -1541,48 +1519,47 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
       <c r="W17" s="1"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="10"/>
-    </row>
-    <row r="18" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X17" s="10"/>
+    </row>
+    <row r="18" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
         <v>16</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="D18" s="11">
         <v>17</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -1590,50 +1567,49 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
       <c r="W18" s="1"/>
-      <c r="X18" s="1"/>
-      <c r="Y18" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X18" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
         <v>17</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>48</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>49</v>
       </c>
       <c r="D19" s="11">
         <v>17</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -1641,20 +1617,19 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
       <c r="W19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X19" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
         <v>18</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D20" s="11">
         <v>27</v>
@@ -1666,17 +1641,17 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
@@ -1686,50 +1661,49 @@
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
       <c r="W20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="21" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X20" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>19</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="5">
+        <v>27</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D21" s="5">
-        <v>27</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F21" s="11"/>
       <c r="G21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
@@ -1737,50 +1711,49 @@
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
-      <c r="X21" s="1"/>
-      <c r="Y21" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="22" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X21" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
         <v>20</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D22" s="11">
         <v>27</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F22" s="11"/>
       <c r="G22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
@@ -1788,20 +1761,19 @@
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X22" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
         <v>21</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>54</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>55</v>
       </c>
       <c r="D23" s="11">
         <v>27</v>
@@ -1809,7 +1781,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="11"/>
       <c r="G23" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -1827,18 +1799,17 @@
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
       <c r="W23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="10"/>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X23" s="10"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
         <v>22</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24" s="11">
         <v>27</v>
@@ -1857,27 +1828,24 @@
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
       <c r="R24" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="S24" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
       <c r="W24" s="1"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="10"/>
-    </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X24" s="10"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
         <v>23</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>57</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>58</v>
       </c>
       <c r="D25" s="11">
         <v>27</v>
@@ -1896,27 +1864,24 @@
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
       <c r="R25" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="S25" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
       <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="10"/>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X25" s="10"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
         <v>24</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D26" s="11">
         <v>27</v>
@@ -1935,27 +1900,24 @@
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
       <c r="R26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="S26" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
       <c r="W26" s="1"/>
-      <c r="X26" s="1"/>
-      <c r="Y26" s="10"/>
-    </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X26" s="10"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A27" s="10">
         <v>25</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D27" s="11">
         <v>27</v>
@@ -1963,12 +1925,12 @@
       <c r="E27" s="12"/>
       <c r="F27" s="11"/>
       <c r="G27" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
@@ -1983,18 +1945,17 @@
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
       <c r="W27" s="1"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="10"/>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X27" s="10"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A28" s="10">
         <v>26</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D28" s="11">
         <v>27</v>
@@ -2005,7 +1966,7 @@
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
@@ -2020,18 +1981,17 @@
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
       <c r="W28" s="1"/>
-      <c r="X28" s="1"/>
-      <c r="Y28" s="10"/>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X28" s="10"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
         <v>27</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D29" s="11">
         <v>27</v>
@@ -2039,10 +1999,10 @@
       <c r="E29" s="12"/>
       <c r="F29" s="11"/>
       <c r="G29" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
@@ -2059,24 +2019,23 @@
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
       <c r="W29" s="1"/>
-      <c r="X29" s="1"/>
-      <c r="Y29" s="10"/>
-    </row>
-    <row r="30" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X29" s="10"/>
+    </row>
+    <row r="30" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
         <v>28</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>64</v>
       </c>
       <c r="D30" s="11">
         <v>42</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F30" s="11"/>
       <c r="G30" s="1"/>
@@ -2084,17 +2043,17 @@
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
@@ -2104,34 +2063,33 @@
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
       <c r="W30" s="1"/>
-      <c r="X30" s="1"/>
-      <c r="Y30" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="31" spans="1:25" ht="90" x14ac:dyDescent="0.2">
+      <c r="X30" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" ht="90" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
         <v>29</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="D31" s="11">
         <v>14</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
@@ -2147,32 +2105,31 @@
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
-      <c r="X31" s="1"/>
-      <c r="Y31" s="10"/>
-    </row>
-    <row r="32" spans="1:25" ht="90" x14ac:dyDescent="0.2">
+      <c r="X31" s="10"/>
+    </row>
+    <row r="32" spans="1:24" ht="90" x14ac:dyDescent="0.2">
       <c r="A32" s="10">
         <v>30</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>68</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>69</v>
       </c>
       <c r="D32" s="11">
         <v>14</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F32" s="12"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
@@ -2188,32 +2145,31 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
-      <c r="X32" s="1"/>
-      <c r="Y32" s="10"/>
-    </row>
-    <row r="33" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X32" s="10"/>
+    </row>
+    <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="10">
         <v>31</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D33" s="11">
         <v>29</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F33" s="12"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
@@ -2229,32 +2185,31 @@
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
-      <c r="X33" s="1"/>
-      <c r="Y33" s="10"/>
-    </row>
-    <row r="34" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X33" s="10"/>
+    </row>
+    <row r="34" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="10">
         <v>32</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D34" s="11">
         <v>29</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F34" s="12"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
@@ -2270,30 +2225,29 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1"/>
-      <c r="X34" s="1"/>
-      <c r="Y34" s="10"/>
-    </row>
-    <row r="35" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X34" s="10"/>
+    </row>
+    <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="10">
         <v>33</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D35" s="11">
         <v>29</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F35" s="12"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
@@ -2309,30 +2263,29 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
-      <c r="X35" s="1"/>
-      <c r="Y35" s="10"/>
-    </row>
-    <row r="36" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X35" s="10"/>
+    </row>
+    <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="10">
         <v>34</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D36" s="11">
         <v>29</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F36" s="12"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
@@ -2348,30 +2301,29 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1"/>
-      <c r="X36" s="1"/>
-      <c r="Y36" s="10"/>
-    </row>
-    <row r="37" spans="1:25" ht="36" x14ac:dyDescent="0.2">
+      <c r="X36" s="10"/>
+    </row>
+    <row r="37" spans="1:24" ht="36" x14ac:dyDescent="0.2">
       <c r="A37" s="10">
         <v>35</v>
       </c>
       <c r="B37" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="D37" s="11">
         <v>14</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F37" s="12"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
@@ -2387,30 +2339,29 @@
       <c r="U37" s="1"/>
       <c r="V37" s="1"/>
       <c r="W37" s="1"/>
-      <c r="X37" s="1"/>
-      <c r="Y37" s="10"/>
-    </row>
-    <row r="38" spans="1:25" ht="36" x14ac:dyDescent="0.2">
+      <c r="X37" s="10"/>
+    </row>
+    <row r="38" spans="1:24" ht="36" x14ac:dyDescent="0.2">
       <c r="A38" s="10">
         <v>36</v>
       </c>
       <c r="B38" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>68</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>69</v>
       </c>
       <c r="D38" s="11">
         <v>14</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F38" s="12"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
@@ -2426,18 +2377,17 @@
       <c r="U38" s="1"/>
       <c r="V38" s="1"/>
       <c r="W38" s="1"/>
-      <c r="X38" s="1"/>
-      <c r="Y38" s="10"/>
-    </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X38" s="10"/>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A39" s="10">
         <v>37</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D39" s="11">
         <v>17</v>
@@ -2456,29 +2406,26 @@
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
       <c r="R39" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="S39" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="T39" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="T39" s="1"/>
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1"/>
-      <c r="X39" s="1"/>
-      <c r="Y39" s="10"/>
-    </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X39" s="10"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A40" s="10">
         <v>38</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D40" s="11">
         <v>17</v>
@@ -2497,29 +2444,26 @@
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
       <c r="R40" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="S40" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="T40" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="T40" s="1"/>
       <c r="U40" s="1"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1"/>
-      <c r="X40" s="1"/>
-      <c r="Y40" s="10"/>
-    </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X40" s="10"/>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A41" s="10">
         <v>39</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D41" s="11">
         <v>25</v>
@@ -2539,30 +2483,29 @@
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
-      <c r="T41" s="1"/>
+      <c r="T41" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="U41" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V41" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="W41" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="X41" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y41" s="10"/>
-    </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+      <c r="X41" s="10"/>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42" s="10">
         <v>40</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="D42" s="11">
         <v>14</v>
@@ -2581,55 +2524,54 @@
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
-      <c r="S42" s="1"/>
-      <c r="T42" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="S42" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T42" s="1"/>
       <c r="U42" s="1"/>
       <c r="V42" s="1"/>
       <c r="W42" s="1"/>
-      <c r="X42" s="1"/>
-      <c r="Y42" s="10"/>
-    </row>
-    <row r="43" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X42" s="10"/>
+    </row>
+    <row r="43" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10">
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D43" s="11">
         <v>17</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R43" s="10"/>
       <c r="S43" s="10"/>
@@ -2637,50 +2579,49 @@
       <c r="U43" s="10"/>
       <c r="V43" s="10"/>
       <c r="W43" s="10"/>
-      <c r="X43" s="10"/>
-      <c r="Y43" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="44" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X43" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="10">
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C44" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D44" s="11">
+        <v>27</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D44" s="11">
-        <v>27</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F44" s="10"/>
       <c r="G44" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
       <c r="O44" s="1"/>
       <c r="P44" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R44" s="10"/>
       <c r="S44" s="10"/>
@@ -2688,50 +2629,49 @@
       <c r="U44" s="10"/>
       <c r="V44" s="10"/>
       <c r="W44" s="10"/>
-      <c r="X44" s="10"/>
-      <c r="Y44" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="45" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X44" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="10">
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D45" s="11">
         <v>17</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F45" s="10"/>
       <c r="G45" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R45" s="10"/>
       <c r="S45" s="10"/>
@@ -2739,50 +2679,49 @@
       <c r="U45" s="10"/>
       <c r="V45" s="10"/>
       <c r="W45" s="10"/>
-      <c r="X45" s="10"/>
-      <c r="Y45" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="46" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X45" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="10">
         <v>44</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C46" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D46" s="11">
+        <v>27</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D46" s="11">
-        <v>27</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F46" s="10"/>
       <c r="G46" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R46" s="10"/>
       <c r="S46" s="10"/>
@@ -2790,50 +2729,49 @@
       <c r="U46" s="10"/>
       <c r="V46" s="10"/>
       <c r="W46" s="10"/>
-      <c r="X46" s="10"/>
-      <c r="Y46" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="47" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X46" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10">
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D47" s="11">
         <v>17</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
       <c r="O47" s="1"/>
       <c r="P47" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R47" s="10"/>
       <c r="S47" s="10"/>
@@ -2841,50 +2779,49 @@
       <c r="U47" s="10"/>
       <c r="V47" s="10"/>
       <c r="W47" s="10"/>
-      <c r="X47" s="10"/>
-      <c r="Y47" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="48" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X47" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10">
         <v>46</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48" s="11">
         <v>27</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F48" s="10"/>
       <c r="G48" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
       <c r="L48" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
       <c r="O48" s="1"/>
       <c r="P48" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R48" s="10"/>
       <c r="S48" s="10"/>
@@ -2892,50 +2829,49 @@
       <c r="U48" s="10"/>
       <c r="V48" s="10"/>
       <c r="W48" s="10"/>
-      <c r="X48" s="10"/>
-      <c r="Y48" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="49" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X48" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="49" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10">
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D49" s="11">
         <v>17</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F49" s="10"/>
       <c r="G49" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
       <c r="O49" s="1"/>
       <c r="P49" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R49" s="10"/>
       <c r="S49" s="10"/>
@@ -2943,50 +2879,49 @@
       <c r="U49" s="10"/>
       <c r="V49" s="10"/>
       <c r="W49" s="10"/>
-      <c r="X49" s="10"/>
-      <c r="Y49" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="50" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X49" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10">
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D50" s="11">
         <v>27</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F50" s="10"/>
       <c r="G50" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
       <c r="L50" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
       <c r="O50" s="1"/>
       <c r="P50" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R50" s="10"/>
       <c r="S50" s="10"/>
@@ -2994,50 +2929,49 @@
       <c r="U50" s="10"/>
       <c r="V50" s="10"/>
       <c r="W50" s="10"/>
-      <c r="X50" s="10"/>
-      <c r="Y50" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="51" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X50" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10">
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D51" s="11">
         <v>17</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F51" s="10"/>
       <c r="G51" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R51" s="10"/>
       <c r="S51" s="10"/>
@@ -3045,50 +2979,49 @@
       <c r="U51" s="10"/>
       <c r="V51" s="10"/>
       <c r="W51" s="10"/>
-      <c r="X51" s="10"/>
-      <c r="Y51" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="52" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X51" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="52" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="10">
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D52" s="11">
         <v>27</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F52" s="10"/>
       <c r="G52" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
       <c r="L52" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
       <c r="O52" s="1"/>
       <c r="P52" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R52" s="10"/>
       <c r="S52" s="10"/>
@@ -3096,26 +3029,25 @@
       <c r="U52" s="10"/>
       <c r="V52" s="10"/>
       <c r="W52" s="10"/>
-      <c r="X52" s="10"/>
-      <c r="Y52" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="53" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X52" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="53" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10">
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D53" s="10">
         <v>42</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F53" s="10"/>
       <c r="G53" s="10"/>
@@ -3123,17 +3055,17 @@
       <c r="I53" s="10"/>
       <c r="J53" s="10"/>
       <c r="K53" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L53" s="1"/>
       <c r="M53" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
@@ -3143,26 +3075,25 @@
       <c r="U53" s="10"/>
       <c r="V53" s="10"/>
       <c r="W53" s="10"/>
-      <c r="X53" s="10"/>
-      <c r="Y53" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="54" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X53" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="54" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="10">
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D54" s="10">
         <v>42</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F54" s="10"/>
       <c r="G54" s="10"/>
@@ -3170,17 +3101,17 @@
       <c r="I54" s="10"/>
       <c r="J54" s="10"/>
       <c r="K54" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L54" s="1"/>
       <c r="M54" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
@@ -3190,26 +3121,25 @@
       <c r="U54" s="10"/>
       <c r="V54" s="10"/>
       <c r="W54" s="10"/>
-      <c r="X54" s="10"/>
-      <c r="Y54" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="55" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X54" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="55" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="10">
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D55" s="10">
         <v>42</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F55" s="10"/>
       <c r="G55" s="10"/>
@@ -3217,17 +3147,17 @@
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
       <c r="K55" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L55" s="1"/>
       <c r="M55" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P55" s="1"/>
       <c r="Q55" s="1"/>
@@ -3237,27 +3167,26 @@
       <c r="U55" s="10"/>
       <c r="V55" s="10"/>
       <c r="W55" s="10"/>
-      <c r="X55" s="10"/>
-      <c r="Y55" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="56" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X55" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="56" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="10">
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D56" s="10"/>
       <c r="E56" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G56" s="10"/>
       <c r="H56" s="10"/>
@@ -3277,47 +3206,46 @@
       <c r="V56" s="10"/>
       <c r="W56" s="10"/>
       <c r="X56" s="10"/>
-      <c r="Y56" s="10"/>
-    </row>
-    <row r="57" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="10">
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D57" s="11">
         <v>17</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F57" s="10"/>
       <c r="G57" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
       <c r="L57" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
       <c r="O57" s="1"/>
       <c r="P57" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q57" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R57" s="10"/>
       <c r="S57" s="10"/>
@@ -3325,50 +3253,49 @@
       <c r="U57" s="10"/>
       <c r="V57" s="10"/>
       <c r="W57" s="10"/>
-      <c r="X57" s="10"/>
-      <c r="Y57" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="58" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X57" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="58" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="10">
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C58" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D58" s="11">
+        <v>27</v>
+      </c>
+      <c r="E58" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D58" s="11">
-        <v>27</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F58" s="10"/>
       <c r="G58" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
       <c r="L58" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M58" s="1"/>
       <c r="N58" s="1"/>
       <c r="O58" s="1"/>
       <c r="P58" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R58" s="10"/>
       <c r="S58" s="10"/>
@@ -3376,50 +3303,49 @@
       <c r="U58" s="10"/>
       <c r="V58" s="10"/>
       <c r="W58" s="10"/>
-      <c r="X58" s="10"/>
-      <c r="Y58" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="59" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X58" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="10">
         <v>57</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D59" s="11">
         <v>17</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F59" s="10"/>
       <c r="G59" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
       <c r="L59" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M59" s="1"/>
       <c r="N59" s="1"/>
       <c r="O59" s="1"/>
       <c r="P59" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q59" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R59" s="10"/>
       <c r="S59" s="10"/>
@@ -3427,50 +3353,49 @@
       <c r="U59" s="10"/>
       <c r="V59" s="10"/>
       <c r="W59" s="10"/>
-      <c r="X59" s="10"/>
-      <c r="Y59" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="60" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X59" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="60" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="10">
         <v>58</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C60" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D60" s="11">
+        <v>27</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D60" s="11">
-        <v>27</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F60" s="10"/>
       <c r="G60" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
       <c r="L60" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
       <c r="O60" s="1"/>
       <c r="P60" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q60" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R60" s="10"/>
       <c r="S60" s="10"/>
@@ -3478,26 +3403,25 @@
       <c r="U60" s="10"/>
       <c r="V60" s="10"/>
       <c r="W60" s="10"/>
-      <c r="X60" s="10"/>
-      <c r="Y60" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="61" spans="1:25" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X60" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="61" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="10">
         <v>59</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D61" s="10">
         <v>42</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F61" s="10"/>
       <c r="G61" s="10"/>
@@ -3505,17 +3429,17 @@
       <c r="I61" s="10"/>
       <c r="J61" s="10"/>
       <c r="K61" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L61" s="1"/>
       <c r="M61" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P61" s="1"/>
       <c r="Q61" s="1"/>
@@ -3525,50 +3449,49 @@
       <c r="U61" s="10"/>
       <c r="V61" s="10"/>
       <c r="W61" s="10"/>
-      <c r="X61" s="10"/>
-      <c r="Y61" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="62" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X61" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="62" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="10">
         <v>60</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D62" s="11">
         <v>17</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F62" s="10"/>
       <c r="G62" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
       <c r="L62" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M62" s="1"/>
       <c r="N62" s="1"/>
       <c r="O62" s="1"/>
       <c r="P62" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q62" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R62" s="10"/>
       <c r="S62" s="10"/>
@@ -3576,50 +3499,49 @@
       <c r="U62" s="10"/>
       <c r="V62" s="10"/>
       <c r="W62" s="10"/>
-      <c r="X62" s="10"/>
-      <c r="Y62" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="63" spans="1:25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X62" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="63" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="10">
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C63" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D63" s="11">
+        <v>27</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D63" s="11">
-        <v>27</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F63" s="10"/>
       <c r="G63" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
       <c r="L63" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M63" s="1"/>
       <c r="N63" s="1"/>
       <c r="O63" s="1"/>
       <c r="P63" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q63" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R63" s="10"/>
       <c r="S63" s="10"/>
@@ -3627,27 +3549,26 @@
       <c r="U63" s="10"/>
       <c r="V63" s="10"/>
       <c r="W63" s="10"/>
-      <c r="X63" s="10"/>
-      <c r="Y63" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="64" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X63" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="64" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="10">
         <v>62</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D64" s="10"/>
       <c r="E64" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G64" s="10"/>
       <c r="H64" s="10"/>
@@ -3667,17 +3588,16 @@
       <c r="V64" s="10"/>
       <c r="W64" s="10"/>
       <c r="X64" s="10"/>
-      <c r="Y64" s="10"/>
-    </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="65" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A65" s="10">
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D65" s="11">
         <v>17</v>
@@ -3685,27 +3605,27 @@
       <c r="E65" s="12"/>
       <c r="F65" s="11"/>
       <c r="G65" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
       <c r="L65" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M65" s="1"/>
       <c r="N65" s="1"/>
       <c r="O65" s="1"/>
       <c r="P65" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q65" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R65" s="1"/>
       <c r="S65" s="1"/>
@@ -3713,50 +3633,49 @@
       <c r="U65" s="1"/>
       <c r="V65" s="1"/>
       <c r="W65" s="1"/>
-      <c r="X65" s="1"/>
-      <c r="Y65" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="66" spans="1:25" ht="18" x14ac:dyDescent="0.2">
+      <c r="X65" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="66" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A66" s="10">
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D66" s="11">
         <v>17</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F66" s="10"/>
       <c r="G66" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J66" s="1"/>
       <c r="K66" s="1"/>
       <c r="L66" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M66" s="1"/>
       <c r="N66" s="1"/>
       <c r="O66" s="1"/>
       <c r="P66" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R66" s="10"/>
       <c r="S66" s="10"/>
@@ -3764,50 +3683,49 @@
       <c r="U66" s="10"/>
       <c r="V66" s="10"/>
       <c r="W66" s="10"/>
-      <c r="X66" s="10"/>
-      <c r="Y66" s="10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="67" spans="1:25" ht="54" x14ac:dyDescent="0.2">
+      <c r="X66" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="67" spans="1:24" ht="54" x14ac:dyDescent="0.2">
       <c r="A67" s="10">
         <v>65</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C67" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D67" s="11">
+        <v>27</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D67" s="11">
-        <v>27</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F67" s="10"/>
       <c r="G67" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
       <c r="L67" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M67" s="1"/>
       <c r="N67" s="1"/>
       <c r="O67" s="1"/>
       <c r="P67" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R67" s="10"/>
       <c r="S67" s="10"/>
@@ -3815,15 +3733,14 @@
       <c r="U67" s="10"/>
       <c r="V67" s="10"/>
       <c r="W67" s="10"/>
-      <c r="X67" s="10"/>
-      <c r="Y67" s="10" t="s">
-        <v>99</v>
+      <c r="X67" s="10" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="F1:T1"/>
+    <mergeCell ref="T1:W1"/>
+    <mergeCell ref="F1:S1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>